<commit_message>
Update chip report site 2026-08-14
</commit_message>
<xml_diff>
--- a/outputs/chip-report/台股盤後籌碼_2026-08-14.xlsx
+++ b/outputs/chip-report/台股盤後籌碼_2026-08-14.xlsx
@@ -582,7 +582,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>本次為 2026-08-14 正式版，已補入 TWSE 與 TAIFEX 官方數據；散戶位階採 45 日中位秩分位，並以小台部位 + 微台部位/5 換算等值口數。</t>
+          <t>本次為 2026-08-14 正式版，已補入 TWSE 與 TAIFEX 官方數據；散戶位階採近45日相對位階（同值取中間排名），並以小台部位 + 微台部位/5 換算等值口數。</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2019,7 @@
       <c r="G112" s="7" t="n"/>
       <c r="I112" s="7" t="inlineStr">
         <is>
-          <t>中位秩百分位 = (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 45 筆。</t>
+          <t>近45日相對位階（同值取中間排名）= (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 45 筆。</t>
         </is>
       </c>
       <c r="J112" s="7" t="n"/>
@@ -2090,21 +2090,21 @@
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
         <is>
-          <t>中位秩百分位 = (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 45 筆。</t>
+          <t>近45日相對位階（同值取中間排名）= (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 45 筆。</t>
         </is>
       </c>
       <c r="B118" s="7" t="n"/>
       <c r="C118" s="7" t="n"/>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>中位秩百分位 = (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 45 筆。</t>
+          <t>近45日相對位階（同值取中間排名）= (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 45 筆。</t>
         </is>
       </c>
       <c r="F118" s="7" t="n"/>
       <c r="G118" s="7" t="n"/>
       <c r="I118" s="7" t="inlineStr">
         <is>
-          <t>中位秩百分位 = (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 45 筆。</t>
+          <t>近45日相對位階（同值取中間排名）= (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 45 筆。</t>
         </is>
       </c>
       <c r="J118" s="7" t="n"/>

</xml_diff>